<commit_message>
A3 M-1 done: ablation baseline, noise floor, perf diagnosis corrected
</commit_message>
<xml_diff>
--- a/tokens_data.xlsx
+++ b/tokens_data.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>prompt</t>
   </si>
@@ -45,6 +45,9 @@
   </si>
   <si>
     <t>date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prompt lost continue </t>
   </si>
 </sst>
 </file>
@@ -363,7 +366,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="125.140625" bestFit="1" customWidth="1"/>
@@ -417,8 +420,16 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C5">
+        <v>37</v>
+      </c>
       <c r="E5" s="1">
-        <v>46270</v>
+        <v>46271</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
A3: narrow the bench degradation to the enemy loop; rule out node churn and editor accumulation
</commit_message>
<xml_diff>
--- a/tokens_data.xlsx
+++ b/tokens_data.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>prompt</t>
   </si>
@@ -38,29 +38,95 @@
     <t>go, after finishing E-5 document everything so I can start a new session due to context finishing and also give prompt for the new session</t>
   </si>
   <si>
-    <t>Continue A2 on the Medieval Horde Defense project.</t>
-  </si>
-  <si>
     <t>weekly</t>
   </si>
   <si>
     <t>date</t>
   </si>
   <si>
-    <t xml:space="preserve">prompt lost continue </t>
+    <t>go, do not reduce enemy number it's not that difficult</t>
+  </si>
+  <si>
+    <t>new_session</t>
+  </si>
+  <si>
+    <t>idk</t>
+  </si>
+  <si>
+    <t>ok document everything, verify a3_plan 's sequencing then ask me to reply go for coding each part. give(not run) cmd for git add and commit for each.</t>
+  </si>
+  <si>
+    <t>go(m-1)</t>
+  </si>
+  <si>
+    <t>go, the commit need not be that big, give cmd for just add everything and commit which part done</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Reply </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>go</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for P-2, or name the rung you want.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Reply </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>go</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for S-1, or name another rung.</t>
+    </r>
+  </si>
+  <si>
+    <t>document everything, document the problem you faced on A3, I will be changing the effort mode in my next prompt, just document and ready a prompt that I can give to opus 5 max</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="2">
@@ -366,13 +432,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="125.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="137.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -383,18 +449,18 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
         <v>5</v>
       </c>
-      <c r="E1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:5">
       <c r="C2">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -411,28 +477,131 @@
         <v>46270</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="1">
-        <v>46270</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5">
+      <c r="E4" s="1"/>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
       <c r="C5">
-        <v>37</v>
+        <v>0</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
       </c>
       <c r="E5" s="1">
         <v>46271</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>27</v>
+      </c>
+      <c r="C6">
+        <v>27</v>
+      </c>
+      <c r="D6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>31</v>
+      </c>
+      <c r="D7">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>11</v>
+      </c>
+      <c r="C8">
+        <v>42</v>
+      </c>
+      <c r="D8">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>50</v>
+      </c>
+      <c r="D9">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10">
         <v>7</v>
+      </c>
+      <c r="C10">
+        <v>57</v>
+      </c>
+      <c r="D10">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>20</v>
+      </c>
+      <c r="C11">
+        <v>77</v>
+      </c>
+      <c r="D11">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12">
+        <v>79</v>
+      </c>
+      <c r="D12">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: density-field flow as the next A3 direction, with research and sources
</commit_message>
<xml_diff>
--- a/tokens_data.xlsx
+++ b/tokens_data.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
   <si>
     <t>prompt</t>
   </si>
@@ -109,6 +109,24 @@
   </si>
   <si>
     <t>document everything, document the problem you faced on A3, I will be changing the effort mode in my next prompt, just document and ready a prompt that I can give to opus 5 max</t>
+  </si>
+  <si>
+    <t>search if any other way this could be done, I want the enemies to flow like fluid simulation like gravity pulling water downward through a maze but this perspective towards the game</t>
+  </si>
+  <si>
+    <t>ultra</t>
+  </si>
+  <si>
+    <t>first document everything, I'm going to start a new session. give prompt for the next session (ready document then ask for "go" to plan it (need to ask go becuase it need to be done using ultra code)</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>not finish</t>
+  </si>
+  <si>
+    <t>try again</t>
   </si>
 </sst>
 </file>
@@ -432,13 +450,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="137.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -455,12 +473,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:6">
       <c r="C2">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -477,10 +495,10 @@
         <v>46270</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:6">
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -494,7 +512,7 @@
         <v>46271</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -508,7 +526,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -522,7 +540,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -536,7 +554,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -550,7 +568,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -564,7 +582,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -578,7 +596,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -592,12 +610,73 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>7</v>
       </c>
       <c r="C13">
         <v>0</v>
+      </c>
+      <c r="E13" s="1">
+        <v>46272</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="C14">
+        <v>50</v>
+      </c>
+      <c r="D14">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>29</v>
+      </c>
+      <c r="C15">
+        <v>79</v>
+      </c>
+      <c r="D15">
+        <v>43</v>
+      </c>
+      <c r="F15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16">
+        <v>100</v>
+      </c>
+      <c r="D16">
+        <v>45</v>
+      </c>
+      <c r="F16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>